<commit_message>
Add architecture and messaging Q&A sheet
Cover Creatio stack (IIS, Redis, DB) and RabbitMQ vs Kafka in
beginner-friendly interview answers.

Co-authored-by: pizhyanov <pizhyanov@gmail.com>
</commit_message>
<xml_diff>
--- a/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
+++ b/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
@@ -12,17 +12,19 @@
     <sheet name="SQL" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="JavaScript" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Creatio_BPMSoft" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Резюме_и_поведение" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Как_готовиться" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="SQL_шпаргалка" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Архитектура_очереди" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Резюме_и_поведение" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Как_готовиться" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SQL_шпаргалка" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C#'!$A$1:$D$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SQL'!$A$1:$D$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'JavaScript'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Creatio_BPMSoft'!$A$1:$D$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Резюме_и_поведение'!$A$1:$D$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Как_готовиться'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Архитектура_очереди'!$A$1:$D$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Резюме_и_поведение'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Как_готовиться'!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -594,76 +596,96 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Резюме_и_поведение</t>
+          <t>Архитектура_очереди</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Разговорная часть</t>
+          <t>IIS, Redis, БД, Rabbit, Kafka</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ЗАРАНЕЕ впишите факты из резюме</t>
+          <t>Схема стенда + сравнение очередей</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Резюме_и_поведение</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Разговорная часть</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ЗАРАНЕЕ впишите факты из резюме</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Как_готовиться</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>План на дни</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Идите сверху вниз, отмечайте статус</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Кандидат</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Владислав Пыжьянов</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="50" customHeight="1">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Стиль файла</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Ответы написаны простым языком «для чайников»: аналогии, шаги, и блок «Что сказать» — готовая короткая формулировка на собеседование.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="50" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Стиль файла</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Ответы написаны простым языком «для чайников»: аналогии, шаги, и блок «Что сказать» — готовая короткая формулировка на собеседование.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Совет</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Не зубрите наизусть длинный текст. Понимайте аналогию → своими словами скажите короткий ответ из блока «Что сказать» → один пример из вашего опыта.</t>
         </is>
@@ -2708,6 +2730,510 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Категория</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Вопрос</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Ответ простыми словами</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Статус (ок/повторить)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="220" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Общая картина</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Из чего состоит типичное приложение Creatio / веб на .NET?</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Представьте ресторан:
+• официант принимает заказ (веб-сервер / IIS / reverse proxy);
+• кухня готовит (приложение Creatio / .NET);
+• холодильник с продуктами (база данных);
+• записка «уже готовили вот это» на стикере (кэш Redis);
+• лента заказов между цехами (очередь Rabbit/Kafka — если есть интеграции).
+Типичный набор для Creatio on-prem / корпоративного стенда:
+1) Браузер пользователя
+2) IIS (или другой web-сервер) — принимает HTTP
+3) Приложение Creatio (.NET) — бизнес-логика, процессы, API
+4) СУБД (MS SQL / PostgreSQL) — главное хранилище
+5) Redis — быстрый кэш и иногда сессии/распределённые штуки
+6) Файловое хранилище (диск / S3-подобное) — вложения
+7) Опционально: планировщик, Elasticsearch, очереди, почтовый сервер
+Что сказать: «Клиент → IIS/web → приложение → БД; рядом Redis-кэш; для интеграций часто очереди; вложения отдельно».</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3" ht="220" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>IIS</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Что такое IIS и зачем он нужен?</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>IIS (Internet Information Services) — веб-сервер Windows от Microsoft.
+Простыми словами: это «дверь в интернет» для сайта/приложения. Браузер стучится на порт 80/443, IIS принимает запрос и отдаёт его приложению Creatio (или статику), потом возвращает ответ.
+Что обычно настраивают:
+• сайт / application pool (пул — «рабочий процесс» приложения);
+• HTTPS-сертификат;
+• привязку к домену;
+• права учётки пула на папки и БД.
+Аналогия: ресепшен офиса — посетитель не бежит сразу в бухгалтерию, сначала проходит через ресепшен.
+Что сказать: «IIS хостит веб-приложение Creatio, раздаёт HTTP/HTTPS, управляет app pool».</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4" ht="194" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>IIS</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Что такое Application Pool?</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Пул приложений — отдельный рабочий процесс Windows, в котором крутится сайт.
+Зачем отдельно: упал один сайт — не обязательно уронил все остальные; можно задать свою учётку, лимиты памяти, автоперезапуск.
+Если пул «засыпает» или часто перезапускается — пользователи видят долгий первый заход или обрыв сессий.
+Что сказать: «Изолированный worker process для сайта; влияет на стабильность и права».</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="220" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>БД</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Какая роль базы данных?</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>БД — главный сейф с данными: контакты, сделки, настройки, права, журналы.
+Creatio без БД не живёт. Всё важное в итоге там (или согласовано с ней).
+Рядом бывают:
+• основная OLTP-база (повседневная работа);
+• иногда реплика/отчётная база для тяжёлых отчётов;
+• бэкапы.
+Что сказать: «СУБД — источник истины; кэш ускоряет чтение, но не заменяет БД».</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="220" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Redis</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Что такое Redis простыми словами?</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Redis — очень быстрое хранилище «ключ → значение» обычно в памяти (RAM).
+Аналогия: не ходить каждый раз в большой архив (БД), а держать частые бумажки на столе под рукой.
+Зачем в приложениях / Creatio-ландшафте:
+• кэш справочников и тяжёлых выборок;
+• сессии / распределённый кэш между несколькими серверами;
+• иногда блокировки, счётчики, pub/sub.
+Важно: данные в Redis могут пропасть при рестарте (зависит от настроек). Туда не кладут единственную копию критичных денег/сделок — только то, что можно заново прочитать из БД.
+Что сказать: «In-memory кэш/ключ-значение; ускоряет чтение; источник истины — БД».</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="220" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Redis</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Как примерно работают с Redis из кода?</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Идея:
+1) Спросили: есть ли в кэше ключ user:123:profile?
+2) Есть — вернули быстро.
+3) Нет — прочитали из БД, положили в Redis с TTL (время жизни), вернули.
+В .NET часто используют StackExchange.Redis: Multiplexer → Database → StringGet/StringSet.
+Правила чайника:
+• ключи именуйте системно (префикс:сущность:id);
+• всегда думайте про TTL и инвалидацию (когда данные в БД изменились — сбросить кэш);
+• не храните огромные объекты без нужды.
+Что сказать: «Cache-aside: сначала Redis, промах → БД → запись в Redis с TTL».</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8" ht="220" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Другие части</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Что ещё часто рядом с приложением?</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>• Reverse proxy / балансировщик (nginx, ARR, HW LB) — если несколько серверов Creatio.
+• Файлы/вложения — диск сервера или объектное хранилище.
+• Почта (SMTP) — уведомления.
+• Elasticsearch / поиск — быстрый полнотекст (если включён в ландшафте).
+• Мониторинг и логи (Windows Event Log, файлы логов, APM).
+• CI/CD и артефакты пакетов.
+• Очереди сообщений (RabbitMQ, Kafka) — интеграции и фоновая обработка.
+Что сказать: перечислите 5–6 блоков и зачем каждый — уже сильный ответ.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="220" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Один сервер и несколько серверов — в чём разница?</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Один сервер: IIS + приложение + иногда даже БД рядом (для учебных стендов).
+Боевой вариант чаще:
+• 2+ сервера приложения за балансировщиком;
+• отдельный SQL;
+• общий Redis, чтобы кэш/сессии видели все ноды;
+• общее файловое хранилище.
+Иначе пользователь попал на сервер A, потом на B — и «пропали» локальные файлы/кэш.
+Что сказать: «При горизонтальном масштабе нужны sticky/общие сессии и общее хранилище».</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10" ht="220" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>RabbitMQ</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Что такое RabbitMQ простыми словами?</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>RabbitMQ — почтовое отделение для программ.
+Одна программа кладёт письмо (сообщение) в очередь, другая забирает и обрабатывает, когда готова. Им не нужно быть онлайн строго в одну секунду.
+Зачем:
+• интеграции («создали заказ → потом отправим в 1С»);
+• не тормозить пользователя долгим действием;
+• сгладить пики нагрузки;
+• повторить обработку, если потребитель упал.
+Ключевые слова: producer (отправитель), queue (очередь), consumer (обработчик), exchange (куда «бросить» и как маршрутизировать).
+Что сказать: «Брокер очередей сообщений; асинхронная связь сервисов».</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="220" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>RabbitMQ</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Как устроена маршрутизация в Rabbit (очень кратко)?</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Продюсер обычно публикует не «сразу в очередь», а в exchange.
+Exchange по правилам кладёт сообщение в одну или несколько очередей.
+Консьюмер читает из очереди.
+Простые типы exchange:
+• direct — точное совпадение ключа маршрутизации;
+• topic — шаблоны вроде order.*;
+• fanout — всем очередям сразу.
+Аналогия: exchange — сортировочный центр, queue — ящик конкретного курьера.
+Что сказать: «Producer → Exchange → Queue → Consumer».</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="220" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>RabbitMQ</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Как работать с RabbitMQ на практике?</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Типовой цикл:
+1) Подняли Rabbit (Docker/сервер), создали exchange/очередь/binding.
+2) В .NET подключились клиентом (например RabbitMQ.Client).
+3) Продюсер: сериализовали JSON → BasicPublish.
+4) Консьюмер: BasicConsume → обработали → Ack (подтвердили).
+5) Если упали без Ack — сообщение можно отдать снова.
+Важные правила:
+• делайте обработку идемпотентной (повтор сообщения не должен дважды списать деньги);
+• ошибочные сообщения — в retry / dead-letter очередь, а не бесконечный цикл;
+• не держите огромные сообщения лучше класть ссылку на файл/Id в БД;
+• следите за ростом очереди (мониторинг).
+Что сказать: «Publish/consume, ack, idempotency, DLQ, мониторинг длины очереди».</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13" ht="220" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Kafka</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Что такое Apache Kafka простыми словами?</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Kafka — большой журнал событий (лог), который читают многие.
+Аналогия: не почтовый ящик «забрал письмо — его больше нет», а лента новостей: события дописываются в конец, разные читатели могут читать с разной скоростью и даже перечитывать историю (в пределах хранения).
+Зачем:
+• много событий (клики, изменения заказа, логи интеграций);
+• несколько систем слушают один поток;
+• нужна высокая пропускная способность и история.
+Слова: producer, topic (тема), partition (часть темы), consumer group, offset (закладка «до куда прочитал»).
+Что сказать: «Распределённый commit-log / event streaming платформа».</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="220" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Kafka</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Как работать с Kafka на практике?</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Типовой цикл:
+1) Создали topic (часто с несколькими partition).
+2) Продюсер пишет события в topic (ключ влияет на то, в какую partition попадёт).
+3) Консьюмер в consumer group читает свою долю partition.
+4) Сдвигает offset, когда обработал.
+В .NET часто Confluent.Kafka: Producer.Produce / Consumer.Consume.
+Правила:
+• думайте событиями («ЗаказОплачен»), а не «вызови вот тот сервис»;
+• один и тот же ключ (например orderId) помогает сохранить порядок внутри partition;
+• обработка должна переживать повтор (at-least-once — частый режим);
+• следите за lag — насколько консьюмер отстаёт от конца топика.
+Что сказать: «Пишем в topic, читаем consumer group’ой, следим за offset/lag, идемпотентность».</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="220" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Сравнение</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>RabbitMQ vs Kafka — в чём разница?</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Очень коротко:
+RabbitMQ — классическая очередь задач/сообщений.
+• сообщение обычно забрали и обработали (как письмо);
+• удобная гибкая маршрутизация (exchange);
+• отлично для команд и задач: «отправь email», «выгрузи в 1С»;
+• проще ментальная модель для многих интеграций CRM.
+Kafka — поток событий / журнал.
+• сообщения долго лежат в логе, их читают многие;
+• сильна на большом потоке событий и replay истории;
+• сложнее эксплуатация (partition, consumer group, retention);
+• отлично для event-driven архитектуры и аналитических пайплайнов.
+Грубая шпаргалка выбора:
+• нужно «сделай задачу воркеру» → чаще Rabbit;
+• нужно «запиши событие, пусть 5 систем слушают и можно переиграть» → чаще Kafka.
+Что сказать: именно эту таблицу различий + 1 пример выбора.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="218" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Сравнение</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Можно ли заменить одно другим?</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Иногда да, часто нет идеально.
+На Rabbit можно строить event-потоки, но история и огромный throughput — не его сильная сторона.
+На Kafka можно делать очереди задач, но для простых RPC-подобных задач Rabbit обычно проще.
+В корпорациях часто живут ОБА: Kafka — шина событий, Rabbit — конкретные рабочие очереди.
+Что сказать: «Инструменты с разным фокусом; выбор от паттерна нагрузки и команды эксплуатации».</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="220" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Creatio</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Где очереди встречаются рядом с Creatio?</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Типовые сценарии:
+• Creatio сохранила заявку → в очередь сообщение → отдельный воркер шлёт в ERP/шину;
+• внешняя система пишет события в Kafka → сервис-адаптер создаёт/обновляет записи в Creatio через API;
+• тяжёлые массовые операции выносят из синхронного save в фон.
+Важно для разработчика Creatio:
+• не делать долгий HTTP внутри сохранения карточки, если можно положить сообщение в очередь;
+• продумать повтор и идемпотентность (Creatio может сохранить, а ответ наружу потеряться);
+• логировать correlation id между CRM и очередью.
+Что сказать: «Очередь развязывает UI Creatio и медленные интеграции; обязательны retry и идемпотентность».</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="162" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Практика</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Что ответить, если спросят: «Расскажите архитектуру вашего стенда»?</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Шаблон ответа:
+«Снаружи пользователи ходят на балансировщик/IIS. Там крутится Creatio на .NET. Данные — в SQL/PostgreSQL. Для ускорения и общей сессии между нодами — Redis. Вложения на файловом/объектном хранилище. Для интеграций — Rabbit или Kafka (у нас был …). Логи и мониторинг отдельно. Пакеты катим dev→test→prod».
+Подставьте, что было у вас по факту. Если чего-то не было — так и скажите честно, но покажите понимание общей схемы.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="156" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Практика</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Мини-сравнение гарантий доставки.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>at-most-once — максимум один раз (можно потерять).
+at-least-once — минимум один раз (можно дубль) — самый частый.
+exactly-once — «ровно один» сложно и дорого, на практике часто делают at-least-once + идемпотентный обработчик.
+Что сказать: «Ориентируюсь на at-least-once и идемпотентность консьюмера».</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
@@ -2985,13 +3511,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3120,12 +3646,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Запишите на диктофон ответ «о себе» и послушайте</t>
+          <t>Пройдите Архитектура_очереди: IIS/Redis/БД + Rabbit vs Kafka</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Убрать воду и запинки</t>
+          <t>Часто спрашивают общую схему стенда</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr"/>
@@ -3138,47 +3664,65 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t>Запишите на диктофон ответ «о себе» и послушайте</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Убрать воду и запинки</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
           <t>Повторите слабые темы (колонка Статус = повторить)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Закрепление</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
+      <c r="D9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Правило</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>На собесе отвечайте схемой: 1) простой смысл 2) короткий термин 3) пример</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Так звучите и понятно, и «по-взрослыму»</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D10"/>
+  <autoFilter ref="A1:D11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Regenerate Excel with reflection vs polymorphism Creatio examples
Co-authored-by: pizhyanov <pizhyanov@gmail.com>
</commit_message>
<xml_diff>
--- a/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
+++ b/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
@@ -18,7 +18,7 @@
     <sheet name="SQL_шпаргалка" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C#'!$A$1:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C#'!$A$1:$D$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SQL'!$A$1:$D$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'JavaScript'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Creatio_BPMSoft'!$A$1:$D$16</definedName>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -851,15 +851,133 @@
     <row r="7" ht="220" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>Рефлексия vs полиморфизм</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Слушатель вроде MscCaseEventListener — это пример рефлексии?</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Коротко: почти, но так говорить на собесе НЕТОЧНО.
+MscCaseEventListener сам по себе — не «пример рефлексии». Это обычный класс-слушатель:
+• наследование от EntityEventListener;
+• override OnInserting / OnUpdating и т.д.;
+• часто атрибут вроде [EntityEventListener(SchemaName = "Case")].
+Рефлексия тут у ПЛАТФОРМЫ, не у вашего кода: при старте/сборке Creatio находит такие классы (часто по атрибутам) и подписывает их на события сущности.
+Как назвать правильно:
+• ваш listener → события / Observer + наследование + hook на жизненный цикл Entity;
+• как Creatio его подцепил → discovery по метаданным/атрибутам, внутри часто рефлексия.
+Что сказать: «Слушатель — обработчик событий сущности. Рефлексию использует платформа, чтобы найти и зарегистрировать классы с атрибутом. В самом listener я пишу обычный C#: override методов, без GetType/Invoke».
+Если сказать «listener — это рефлексия» — могут поправить. Если сказать «платформа через атрибуты и рефлексию регистрирует listener’ы» — правильно.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8" ht="220" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Полиморфизм в Creatio</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Пример полиморфизма в Creatio?</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Смысл полиморфизма: один и тот же «разъём», разное поведение.
+Пример 1. EntityEventListener
+Базовый класс говорит: есть OnInserting / OnUpdating. Ваши классы делают разное:
+public class MscCaseEventListener : EntityEventListener {
+  public override void OnInserting(...) {
+    // для Case: проверить обязательные поля
+  }
+}
+public class MscContactEventListener : EntityEventListener {
+  public override void OnInserting(...) {
+    // для Contact: проставить источник лида
+  }
+}
+Платформа вызывает один и тот же метод жизненного цикла, а срабатывает ВАША реализация. Это полиморфизм (virtual/override).
+Пример 2. Клиентские схемы JS
+Родительская страница имеет save(). Ваша replacing-схема делает save по-своему и при необходимости зовёт this.callParent(arguments).
+Что сказать: «Полиморфизм — когда платформа вызывает общий метод, а поведение подставляется классом схемы/listener’а».</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="220" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Рефлексия в Creatio</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Пример рефлексии в Creatio?</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Смысл рефлексии: узнать тип/члены во время работы и вызвать их по имени/метаданным.
+Вы сами редко пишете GetType(), но платформа — да.
+Пример 1. Как платформа находит listener
+Классы с атрибутом [EntityEventListener(SchemaName = "Case")]. Creatio сканирует сборки, читает атрибуты и регистрирует обработчики — это рефлексия/метаданные.
+Пример 2. Работа с Entity «универсально»
+entity.SetColumnValue("Name", "Иван");
+var status = entity.GetTypedColumnValue&lt;Guid&gt;("StatusId");
+Снаружи это API Entity, внутри платформа по имени колонки находит поле схемы. На собесе: «прикладной след метаданных — обращение к полям по имени, а не только через жёсткие свойства класса».
+Пример 3. «Ручная» рефлексия (редко в прикладном коде)
+var type = Type.GetType("Terrasoft.Configuration.MyService, MyPackage");
+var service = Activator.CreateInstance(type);
+type.GetMethod("Run")?.Invoke(service, null);
+В Creatio так обычно не пишут без нужды — лучше явный класс/интерфейс.
+Что сказать: «Рефлексия у платформы: атрибуты listener’ов и метаданные схемы; в моём коде чаще Entity по имени колонки, а не ручной Invoke».</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10" ht="220" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Рефлексия vs полиморфизм</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Как не перепутать рефлексию и полиморфизм? (шпаргалка)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Вопрос полиморфизма: какое поведение подставить?
+Creatio: override OnInserting, callParent, разные listener’ы.
+Аналогия: разные пульты с кнопкой «Сохранить».
+Вопрос рефлексии: что это за тип и какие у него члены?
+Creatio: поиск классов по атрибутам, работа со схемой/полями по имени.
+Аналогия: открыть инструкцию к неизвестной коробке и нажать кнопку по названию.
+Готовый ответ на собесе:
+«Полиморфизм — мои EntityEventListener с разным OnInserting. Рефлексия — сторона платформы: находит listener’ы по атрибутам и работает с метаданными схемы; в прикладном коде я чаще вижу это как работу с Entity/колонками по имени, а не как ручной Invoke».</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="220" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>Интерфейсы</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Что такое интерфейс? Объясните как чайнику.</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Интерфейс — это договор.
 Пример: розетка. Неважно, чайник это или зарядка — если вилка подходит под стандарт, включится. Интерфейс говорит: «умеешь вот эти действия» — а КАК именно умеешь, каждый класс решает сам.
@@ -872,20 +990,20 @@
 Что сказать: «Контракт без реализации. Нужен для гибкости и подмены реализаций».</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="220" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="220" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Интерфейсы</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Зачем писать код через интерфейсы?</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Чтобы не привязываться к одной конкретной реализации.
 Плохо: класс жёстко создаёт new SmtpClient() внутри себя.
@@ -898,20 +1016,20 @@
 В Creatio та же мысль: сервисы, обработчики, процессы — лучше не писать «лапшу» в одном месте.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="170" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13" ht="170" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Интерфейсы</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Что такое явное (explicit) определение интерфейса?</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Обычная реализация: метод виден на самом классе.
 Явная: метод виден только если смотреть на объект «как на интерфейс».
@@ -919,40 +1037,40 @@
 Что сказать коротко: «Метод доступен только через приведение к интерфейсу».</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="142" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="142" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Интерфейсы</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Может ли в интерфейсе быть готовый код?</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Раньше — нет, только «что уметь», без «как».
 С C# 8+ можно писать default-методы (готовая реализация прямо в интерфейсе).
 На собесе достаточно: «Классически интерфейс — контракт. В новых версиях C# добавили default interface methods, но в корпоративном коде ими не злоупотребляют».</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11" ht="220" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="220" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>ООП</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>SOLID — что это простыми словами?</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Пять правил «чтобы код не превратился в кашу»:
 S — один класс = одна задача. Не мешайте сохранение записи и отправку письма в одном монстре.
@@ -964,20 +1082,20 @@
 Что сказать: перечислите буквы своими словами + 1 пример — этого хватает.</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12" ht="194" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="194" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ООП</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Инкапсуляция, наследование, полиморфизм — по-простому.</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Инкапсуляция — прячем внутренности. Как пульт: кнопки снаружи, схема внутри.
 Наследование — «ребёнок» забирает общее у «родителя» и добавляет своё.
@@ -986,20 +1104,20 @@
 Что сказать: три определения + короткий пример из жизни или из CRM.</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13" ht="180" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="180" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>ООП</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>virtual, override, new — в чём разница?</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>virtual — «этот метод можно переопределить в наследнике».
 override — «я реально переопределяю поведение родителя» (настоящий полиморфизм).
@@ -1008,20 +1126,20 @@
 Что сказать: «Для полиморфизма нужны virtual/override. new лучше не использовать без нужды».</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="204" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="204" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Типы</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Value type и Reference type — чем отличаются?</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Value type (int, bool, DateTime, struct) — «само значение». Копируете переменную — копируете содержимое.
 Reference type (class, string, массивы) — «ссылка на объект в памяти». Копируете переменную — копируете адрес, оба смотрят на один объект (кроме string: строки нельзя менять, поэтому ощущение другое).
@@ -1029,20 +1147,20 @@
 Что сказать: разница в копировании и хранении + пример int vs класс Entity.</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15" ht="170" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="170" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Типы</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Что такое null и int?</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Обычный int нулём быть не может — всегда число.
 int? (nullable) — «либо число, либо пусто».
@@ -1050,20 +1168,20 @@
 Что сказать: «Nullable value types и проверки на null обязательны, особенно при чтении из БД».</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16" ht="180" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="180" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Коллекции</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>List, Dictionary, HashSet — когда что?</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>List — список по порядку, «первый, второй, третий». Как очередь номеров.
 Dictionary — словарь «ключ → значение». Быстро найти по Id. Как телефонная книга.
@@ -1072,20 +1190,20 @@
 Что сказать: выбираю структуру под задачу: порядок / поиск по ключу / уникальность.</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17" ht="220" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21" ht="220" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>LINQ</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Что такое LINQ простыми словами?</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Удобный способ спросить у коллекции: «дай где…», «преврати в…», «посчитай…».
 Where — отфильтровать.
@@ -1095,20 +1213,20 @@
 Что сказать: «LINQ — запросы к данным в коде. Where/Select, помнить про deferred execution».</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18" ht="220" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22" ht="220" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>async/await</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Что такое async/await без сложных слов?</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Когда программа ждёт ответ из интернета или БД, глупо просто «замирать и ничего не делать».
 async/await — способ сказать: «пойду ждать ответ, а поток пусть пока займётся другим».
@@ -1118,20 +1236,20 @@
 Что сказать: «Асинхронность для I/O. await не блокирует поток как Sleep».</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="208" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23" ht="208" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Исключения</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Как правильно работать с ошибками (try/catch)?</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>try — пробуем опасное.
 catch — ловим то, что умеем обработать.
@@ -1141,20 +1259,20 @@
 В Creatio: пользователю — ясно «почему не сохранилось», в лог — подробности для разработчика.</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="170" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="170" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>IDisposable</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Зачем using и Dispose?</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Некоторые вещи нужно обязательно закрыть: файл, соединение с БД.
 using сам закроет даже если случилась ошибка.
@@ -1162,20 +1280,20 @@
 Что сказать: «IDisposable + using для детерминированного освобождения ресурсов».</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21" ht="170" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="170" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Строки</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Почему StringBuilder, а не string + string в цикле?</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>string нельзя «дописать» — каждый раз создаётся новая строка.
 В цикле из тысяч сложений это тормозит и жрёт память.
@@ -1183,40 +1301,40 @@
 Что сказать: «string immutable; для частых конкатенаций — StringBuilder».</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22" ht="156" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="156" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Generics</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Что такое generics?</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Шаблон с типом-параметром: List&lt;int&gt;, List&lt;string&gt; — один код, разные типы, без каши из object.
 Плюс: типобезопасность (компилятор ругается раньше) и без лишних упаковок для чисел.
 Что сказать: «Обобщения дают переиспользование без потери типов».</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23" ht="156" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27" ht="156" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>События</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>delegate, event, Action, Func — кратко.</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Делегат — «ссылка на метод».
 Action / Func — готовые удобные делегаты (сделай что-то / сделай и верни).
@@ -1224,20 +1342,20 @@
 Аналогия: event — кнопка звонка в подъезд; жильцы подписываются на «кто-то звонит».</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24" ht="220" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28" ht="220" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Creatio C#</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Как в Creatio работать с записью (Entity)?</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Простыми шагами:
 1) Берём подключение пользователя (UserConnection) — «я работаю от имени системы/юзера».
@@ -1249,20 +1367,20 @@
 Что сказать: «Через Entity/UserConnection: Fetch → SetColumnValue → Save; учитываю права».</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr"/>
-    </row>
-    <row r="25" ht="220" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29" ht="220" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Creatio C#</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>EntitySchemaQuery или голый SQL — что выбрать?</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>ESQ — «правильный» способ платформы спросить данные: учитывает права, схемы, безопаснее.
 Прямой SQL — когда очень сложный отчёт или нужно быстрее/гибче, но:
@@ -1273,20 +1391,20 @@
 Что сказать именно так — звучит зрело.</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26" ht="220" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30" ht="220" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Creatio C#</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Что такое EntityEventListener?</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Это «сторож» на события записи: перед/после добавления, изменения, удаления.
 Примеры:
@@ -1294,23 +1412,24 @@
 • при создании контакта дописать поле «Источник».
 Важно: не устраивать вечный цикл Save → событие → снова Save.
 Тяжёлые внешние вызовы в событии — осторожно (может тормозить сохранение).
+На собесе не путайте с рефлексией: сам listener — это полиморфизм (override OnInserting). Рефлексию использует платформа, чтобы НАЙТИ ваш класс по атрибуту. Подробнее — лист C#, блок «Рефлексия vs полиморфизм».
 Что сказать: «Подписка на жизненный цикл Entity для валидаций и побочной логики».</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr"/>
-    </row>
-    <row r="27" ht="194" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31" ht="194" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Creatio C#</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Процесс Creatio или C#-код — когда что?</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Процесс (визуальный BPM) — когда шаги понятны бизнесу: согласование, письмо, ждать 2 дня, развилка.
 C# — когда сложный алгоритм, интеграция, производительность, много переиспользования.
@@ -1318,20 +1437,20 @@
 Что сказать: «Low-code для оркестрации, код для сложной логики».</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28" ht="208" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32" ht="208" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Практика</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Как искать баг «поле иногда не сохраняется»?</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Не гадайте — идите по чеклисту:
 1) Воспроизвести под той же ролью, что у пользователя.
@@ -1342,20 +1461,20 @@
 Что сказать: показать системный подход. Это ценится больше, чем «я сразу знаю причину».</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr"/>
-    </row>
-    <row r="29" ht="184" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33" ht="184" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Делегаты vs интерфейсы</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Когда делегат, когда интерфейс?</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Делегат/Action — одна простая реакция: «когда готово — вызови вот это».
 Интерфейс — набор связанных умений и нормальный объект с жизнью.
@@ -1364,40 +1483,40 @@
 Что сказать: «Делегат для колбэка, интерфейс для зависимости с несколькими операциями».</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr"/>
-    </row>
-    <row r="30" ht="156" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34" ht="156" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Equals</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Зачем Equals и GetHashCode вместе?</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Если кладёте объекты в Dictionary/HashSet как ключи, сравнение и хеш должны быть согласованы: равные объекты → одинаковый hash.
 В CRM обычно равенство записей — по Id (Guid), а не по всем полям.
 Что сказать: «Пара должна быть согласована; для Entity сравниваем по Id».</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr"/>
-    </row>
-    <row r="31" ht="180" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35" ht="180" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Потоки</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Что такое race condition и lock?</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Race — два потока одновременно портят общие данные, как два человека правят один Excel.
 lock — «сейчас работает только один, остальные подождут».
@@ -1405,10 +1524,10 @@
 Что сказать: «Гонка за общее состояние; синхронизация через lock/concurrent-коллекции; static mutable — риск».</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D31"/>
+  <autoFilter ref="A1:D35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add clear ESQ vs Select comparison for Creatio interviews
Explain EntitySchemaQuery versus Core.DB Select/Insert/Update in
beginner-friendly terms on C# and merged Creatio sheets.

Co-authored-by: pizhyanov <pizhyanov@gmail.com>
</commit_message>
<xml_diff>
--- a/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
+++ b/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
@@ -24,7 +24,7 @@
     <sheet name="Ваши_WEB" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C#'!$A$1:$D$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C#'!$A$1:$D$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SQL'!$A$1:$D$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'JavaScript'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Creatio_BPMSoft'!$A$1:$D$16</definedName>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr"/>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="200" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>CR</t>
@@ -5756,7 +5756,13 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>(ESQ, классы Select, Insert, Update и т.д., Entity-model)</t>
+          <t>Клиент (JS): в основном ESQ, сервисы (ServiceHelper), иногда OData-подобные вызовы.
+Сервер (C#): Entity, ESQ, Select/Insert/Update/Delete (Core.DB), редко голый SQL.
+Отличие ESQ и Select:
+• ESQ — схемы Creatio + права;
+• Select — SQL-конструктор ближе к БД, гибче, осторожнее с правами.
+Что сказать: «Клиент — ESQ/сервисы; сервер — Entity/ESQ/Core.DB Select».
+[ответ дополнен]</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -7161,7 +7167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7860,10 +7866,53 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>Отличия ESQ и Select (классы Select/Insert/Update)?</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>В Creatio на сервере есть ДВА разных «слоя» работы с данными — их часто путают.
+1) EntitySchemaQuery (ESQ)
+• Работает на уровне СХЕМ объектов Creatio (Contact, Account…).
+• Учитывает права доступа, локализацию, многие правила платформы.
+• Удобен для обычных выборок «по-бизнесовому».
+• Есть и на сервере (C#), и на клиенте (JS).
+• Аналогия: заказать блюдо через официанта ресторана Creatio — он знает меню и правила.
+2) Select / Insert / Update / Delete (Terrasoft.Core.DB)
+• Это конструкторы SQL ближе к «голому» запросу, но через API платформы (не всегда руками пишете текст SQL).
+• Гибче и иногда быстрее для сложных запросов.
+• Права записей сами по себе могут НЕ применяться так, как в ESQ — вы ближе к уровню таблиц БД.
+• Обычно только сервер (C#).
+• Аналогия: пройти на кухню и самому собрать ингредиенты — больше контроля, больше ответственности.
+3) Entity (Fetch/Save)
+• Одна запись: прочитал → поменял поля → Save.
+• Для CRUD одной сущности.
+4) Голый SQL / хранимки
+• Ещё ниже уровнем; только когда без этого никак.
+Когда что:
+• Обычная бизнес-выборка с правами → ESQ.
+• Сложный SQL-образный запрос на сервере, отчёт, тонкая оптимизация → Select/Update…
+• Одна запись → Entity.
+Бонус: у ESQ можно получить SQL-текст:
+esq.GetSelectQuery(UserConnection).GetSqlText()
+— то есть ESQ внутри часто превращается в Select/SQL.
+Что сказать: «ESQ — объектный запрос платформы с правами; Select/Insert/Update — более низкоуровневые SQL-конструкторы Core.DB; Entity — работа с одной записью».</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31" ht="220" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Creatio C#</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
           <t>Что такое EntityEventListener?</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Это «сторож» на события записи: перед/после добавления, изменения, удаления.
 Примеры:
@@ -7875,20 +7924,20 @@
 Что сказать: «Подписка на жизненный цикл Entity для валидаций и побочной логики».</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr"/>
-    </row>
-    <row r="31" ht="194" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32" ht="194" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Creatio C#</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Процесс Creatio или C#-код — когда что?</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Процесс (визуальный BPM) — когда шаги понятны бизнесу: согласование, письмо, ждать 2 дня, развилка.
 C# — когда сложный алгоритм, интеграция, производительность, много переиспользования.
@@ -7896,20 +7945,20 @@
 Что сказать: «Low-code для оркестрации, код для сложной логики».</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32" ht="208" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33" ht="208" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Практика</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Как искать баг «поле иногда не сохраняется»?</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Не гадайте — идите по чеклисту:
 1) Воспроизвести под той же ролью, что у пользователя.
@@ -7920,20 +7969,20 @@
 Что сказать: показать системный подход. Это ценится больше, чем «я сразу знаю причину».</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr"/>
-    </row>
-    <row r="33" ht="184" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34" ht="184" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Делегаты vs интерфейсы</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Когда делегат, когда интерфейс?</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Делегат/Action — одна простая реакция: «когда готово — вызови вот это».
 Интерфейс — набор связанных умений и нормальный объект с жизнью.
@@ -7942,40 +7991,40 @@
 Что сказать: «Делегат для колбэка, интерфейс для зависимости с несколькими операциями».</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr"/>
-    </row>
-    <row r="34" ht="156" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35" ht="156" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Equals</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Зачем Equals и GetHashCode вместе?</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Если кладёте объекты в Dictionary/HashSet как ключи, сравнение и хеш должны быть согласованы: равные объекты → одинаковый hash.
 В CRM обычно равенство записей — по Id (Guid), а не по всем полям.
 Что сказать: «Пара должна быть согласована; для Entity сравниваем по Id».</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35" ht="180" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36" ht="180" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Потоки</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Что такое race condition и lock?</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Race — два потока одновременно портят общие данные, как два человека правят один Excel.
 lock — «сейчас работает только один, остальные подождут».
@@ -7983,10 +8032,10 @@
 Что сказать: «Гонка за общее состояние; синхронизация через lock/concurrent-коллекции; static mutable — риск».</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D35"/>
+  <autoFilter ref="A1:D36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Expand SQL answer for views, stored procs, triggers, functions
Replace short stub with beginner-friendly comparison and add the
same topic to the main SQL study sheet.

Co-authored-by: pizhyanov <pizhyanov@gmail.com>
</commit_message>
<xml_diff>
--- a/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
+++ b/Creatio_Interview/Creatio_Interview_QA_Pyzhyanov.xlsx
@@ -25,7 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'C#'!$A$1:$D$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SQL'!$A$1:$D$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SQL'!$A$1:$D$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'JavaScript'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Creatio_BPMSoft'!$A$1:$D$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Архитектура_очереди'!$A$1:$D$19</definedName>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5178,18 +5178,15 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>CREATE VIEW название_представления [(столбец_1, столбец_2, ....)]
-AS выражение_SELECT
-CREATE PROCEDURE [dbo].[sp_InsertUser]
-    @name nvarchar(50),
-    @age int
-AS
-    INSERT INTO Users (Name, Age)
-    VALUES (@name, @age)
-    SELECT SCOPE_IDENTITY()
-GO
-Функция имеет возвращаемый тип и возвращает значение ,не имеет выходных аргументов, вызов хранимой процедуры из функции невозможно, SELECT возможен.
-Хранимая процедура не имеет возвращаемого типа, но имеет выходные аргументы, хранимая процедура имеет и входные, и выходные аргументы, Select не возможен</t>
+          <t>VIEW (представление) — сохранённый SELECT «как виртуальная таблица». Обычно данные сам не хранит, при каждом обращении выполняет запрос. Зачем: упростить сложный JOIN, скрыть лишние поля, дать готовую выборку.
+Хранимая процедура («хранимка») — программа внутри БД: параметры, несколько шагов, может читать и менять данные (SELECT/INSERT/UPDATE/DELETE), транзакции. Вызов: EXEC dbo.MyProc @id = 1.
+Триггер — код, который БД запускает автоматически при INSERT/UPDATE/DELETE. Пример: при удалении писать в журнал аудита. Минус: логика скрыта, легко получить рекурсию и тормоза. В Creatio бизнес-логику чаще держат в C#/процессах, не в триггерах.
+Процедура vs функция:
+• Функция должна вернуть значение (число/строку/таблицу) и обычно вызывается из SELECT: SELECT dbo.GetName(@id). В классических функциях SQL Server нельзя свободно менять таблицы.
+• Процедура вызывается через EXEC, может менять данные, иметь OUTPUT-параметры и несколько наборов строк; её нельзя просто подставить в SELECT как скалярную функцию.
+Шпаргалка: VIEW = готовая выборка; процедура = «сделай работу»; функция = «посчитай и верни»; триггер = «сработай сам при изменении».
+Что сказать: именно эту шпаргалку + 1 пример на каждый объект.
+[ответ дополнен]</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -8046,7 +8043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8460,38 +8457,63 @@
       </c>
       <c r="D18" s="5" t="inlineStr"/>
     </row>
-    <row r="19" ht="146" customHeight="1">
+    <row r="19" ht="220" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Объекты БД</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Представления, хранимки, триггеры. Отличия процедур от функций?</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>VIEW (представление) — сохранённый SELECT «как виртуальная таблица». Обычно данные сам не хранит, при каждом обращении выполняет запрос. Зачем: упростить сложный JOIN, скрыть лишние поля, дать готовую выборку.
+Хранимая процедура («хранимка») — программа внутри БД: параметры, несколько шагов, может читать и менять данные (SELECT/INSERT/UPDATE/DELETE), транзакции. Вызов: EXEC dbo.MyProc @id = 1.
+Триггер — код, который БД запускает автоматически при INSERT/UPDATE/DELETE. Пример: при удалении писать в журнал аудита. Минус: логика скрыта, легко получить рекурсию и тормоза. В Creatio бизнес-логику чаще держат в C#/процессах, не в триггерах.
+Процедура vs функция:
+• Функция должна вернуть значение (число/строку/таблицу) и обычно вызывается из SELECT: SELECT dbo.GetName(@id). В классических функциях SQL Server нельзя свободно менять таблицы.
+• Процедура вызывается через EXEC, может менять данные, иметь OUTPUT-параметры и несколько наборов строк; её нельзя просто подставить в SELECT как скалярную функцию.
+Шпаргалка: VIEW = готовая выборка; процедура = «сделай работу»; функция = «посчитай и верни»; триггер = «сработай сам при изменении».
+Что сказать: именно эту шпаргалку + 1 пример на каждый объект.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="146" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Безопасность</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Что такое SQL injection?</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Злоумышленник вписывает в поле ввода кусок SQL и ломает запрос.
 Защита: никогда не склеивать SQL строкой из текста пользователя. Только параметры.
 Что сказать: «Параметризованные запросы, никаких конкатенаций пользовательского ввода».</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="156" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21" ht="156" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>UNION</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>UNION и JOIN — не путать.</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>JOIN — добавить колонки справа (вширь).
 UNION — поставить наборы строк друг под другом (вниз), структура колонок должна совпадать.
@@ -8499,20 +8521,20 @@
 Что сказать: горизонтальная связь vs вертикальное объединение.</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21" ht="180" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22" ht="180" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Creatio SQL</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Особенности БД Creatio для новичка?</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>• Много системных таблиц.
 • Часто soft delete (IsDeleted), а не физическое удаление.
@@ -8521,20 +8543,20 @@
 Что сказать: «Метаданные через конфигурацию; SQL — осознанно; помнить про права и soft delete».</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22" ht="174" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23" ht="174" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Практика</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Посчитать контакты по каждому аккаунту.</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>SELECT a.Name, COUNT(c.Id) AS Cnt
 FROM Account a
@@ -8544,20 +8566,20 @@
 Условия на контакт лучше в ON, не в WHERE.</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23" ht="174" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="174" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Практика</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Найти дубли email.</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>SELECT Email, COUNT(*) AS Cnt
 FROM Contact
@@ -8567,29 +8589,29 @@
 Что сказать: GROUP BY + HAVING COUNT(*) &gt; 1 — классика собеса.</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24" ht="108" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="108" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Практика</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Чем опасен SELECT *?</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Тащите лишние поля, больше сети/памяти, хрупкий код (добавили колонку — всё поехало), сложнее покрывать индексом.
 Что сказать: «Беру только нужные колонки».</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D24"/>
+  <autoFilter ref="A1:D25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>